<commit_message>
Vòng sửa QA: chặn dòng có trong sheet Hủy, khoá áp dụng lô nhập, kiểm mã trùng mọi tài khoản, ẩn khoản thu; id sai dạng trả 404, whitelist sắp xếp, CSRF chặt hơn; demo-feed qua lõi, service connector riêng
</commit_message>
<xml_diff>
--- a/fixtures/demo-lich-dat-phong.xlsx
+++ b/fixtures/demo-lich-dat-phong.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="186">
   <si>
     <t>DANH SÁCH LỊCH ĐẶT PHÒNG (DEMO — dữ liệu giả)</t>
   </si>
@@ -517,6 +517,21 @@
   </si>
   <si>
     <t>+36 00 000 0027</t>
+  </si>
+  <si>
+    <t>Khách Demo 28</t>
+  </si>
+  <si>
+    <t>Booking 460,86e TM</t>
+  </si>
+  <si>
+    <t>10 tháng 3 2027</t>
+  </si>
+  <si>
+    <t>12 tháng 3 2027</t>
+  </si>
+  <si>
+    <t>+36 00 000 0028</t>
   </si>
   <si>
     <t>DANH SÁCH LỊCH ĐẶT PHÒNG (DEMO)</t>
@@ -936,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2028,6 +2043,44 @@
       </c>
       <c r="N29" t="s">
         <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" t="s">
+        <v>168</v>
+      </c>
+      <c r="E30" t="s">
+        <v>74</v>
+      </c>
+      <c r="F30">
+        <v>1000000028</v>
+      </c>
+      <c r="G30" t="s">
+        <v>169</v>
+      </c>
+      <c r="H30" t="s">
+        <v>170</v>
+      </c>
+      <c r="I30">
+        <v>2</v>
+      </c>
+      <c r="J30" t="s">
+        <v>21</v>
+      </c>
+      <c r="K30">
+        <v>2</v>
+      </c>
+      <c r="N30" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2046,7 +2099,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -2086,7 +2139,7 @@
         <v>8</v>
       </c>
       <c r="I2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -2095,7 +2148,7 @@
         <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -2133,7 +2186,7 @@
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -2159,7 +2212,7 @@
         <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -2171,7 +2224,7 @@
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -2182,7 +2235,7 @@
         <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
@@ -2194,10 +2247,10 @@
         <v>1000000099</v>
       </c>
       <c r="G5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H5" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -2209,7 +2262,7 @@
         <v>2</v>
       </c>
       <c r="L5" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2269,37 +2322,37 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F2">
-        <v>1000000001</v>
+        <v>1000000003</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2" t="s">
         <v>21</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2" t="s">
         <v>128</v>
@@ -2325,13 +2378,13 @@
         <v>109</v>
       </c>
       <c r="F3" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="G3" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -2359,18 +2412,18 @@
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B3" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>

</xml_diff>